<commit_message>
Excel attachment: store unrounded values so totals are exact
data-verifier failed the first .xlsx: totals summed cells pre-rounded to 2
decimals (Hyderabad 90+ off 0.027 MT), one row showed over-30 > on-hand, and
a note described a "0" that displayed as "-". Cells now hold exact values
(each asserted to round to the verified CSV), zeros show 0.00, and the
rounding caveat note is gone. Re-verification pending.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVVKmwQKKV189dev92iFna
</commit_message>
<xml_diff>
--- a/reports/SKU-Ageing-over-30d-2026-10-26.xlsx
+++ b/reports/SKU-Ageing-over-30d-2026-10-26.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="124">
   <si>
     <t xml:space="preserve">Stock over 30 days, by plant (MT) - as of 26-Oct-2026</t>
   </si>
@@ -384,7 +384,7 @@
     <t xml:space="preserve">The three age columns split each SKU's over-30-day tonnage by bracket; "Over 30 days" is their sum.</t>
   </si>
   <si>
-    <t xml:space="preserve">"Sold since 19-Oct" = tonnes of that SKU's aged stock invoiced since last week's mail. 0 (red) = nothing moved; "new" = crossed 30 days this week.</t>
+    <t xml:space="preserve">"Sold since 19-Oct" = tonnes of that SKU's aged stock invoiced since last week's mail. 0.00 (red) = nothing moved; "new" = crossed 30 days this week.</t>
   </si>
   <si>
     <t xml:space="preserve">Sells to: Hyderabad and Lepakshi serve South distributors; NPMD and Tapi serve West.</t>
@@ -394,9 +394,6 @@
   </si>
   <si>
     <t xml:space="preserve">SKUs that sold out completely since 19-Oct are not listed (no stock over 30 days left), so "Sold since 19-Oct" is not totalled here. Total sold from last week's aged stock: 87.9 MT (see the email).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Totals add rows already rounded to 2 decimals, so they can differ by 0.1 MT from the email (e.g. 757.34 here, 757.4 there).</t>
   </si>
   <si>
     <t xml:space="preserve">Figures come from the system. Please check availability with the plant before committing quantities.</t>
@@ -406,9 +403,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00;\-#,##0.00;\-"/>
+    <numFmt numFmtId="166" formatCode="#,##0.00"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -653,11 +651,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1061,19 +1059,19 @@
       </c>
       <c r="D4" s="5" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A4,'Over 30 days'!$E$5:$E$92)</f>
-        <v>488.19</v>
+        <v>488.218343974613</v>
       </c>
       <c r="E4" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A4,'Over 30 days'!$F$5:$F$92)</f>
-        <v>187.9</v>
+        <v>187.902516650575</v>
       </c>
       <c r="F4" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A4,'Over 30 days'!$G$5:$G$92)</f>
-        <v>50.49</v>
+        <v>50.4890326755662</v>
       </c>
       <c r="G4" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A4,'Over 30 days'!$H$5:$H$92)</f>
-        <v>249.8</v>
+        <v>249.826794648472</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1089,11 +1087,11 @@
       </c>
       <c r="D5" s="5" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A5,'Over 30 days'!$E$5:$E$92)</f>
-        <v>156.85</v>
+        <v>156.858534368</v>
       </c>
       <c r="E5" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A5,'Over 30 days'!$F$5:$F$92)</f>
-        <v>156.85</v>
+        <v>156.858534368</v>
       </c>
       <c r="F5" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A5,'Over 30 days'!$G$5:$G$92)</f>
@@ -1117,11 +1115,11 @@
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A6,'Over 30 days'!$E$5:$E$92)</f>
-        <v>36.69</v>
+        <v>36.6708372</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A6,'Over 30 days'!$F$5:$F$92)</f>
-        <v>36.69</v>
+        <v>36.6708372</v>
       </c>
       <c r="F6" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A6,'Over 30 days'!$G$5:$G$92)</f>
@@ -1145,11 +1143,11 @@
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A7,'Over 30 days'!$E$5:$E$92)</f>
-        <v>75.61</v>
+        <v>75.6026841</v>
       </c>
       <c r="E7" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A7,'Over 30 days'!$F$5:$F$92)</f>
-        <v>75.61</v>
+        <v>75.6026841</v>
       </c>
       <c r="F7" s="6" t="n">
         <f aca="false">SUMIF('Over 30 days'!$B$5:$B$92,A7,'Over 30 days'!$G$5:$G$92)</f>
@@ -1171,19 +1169,19 @@
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">SUM(D4:D7)</f>
-        <v>757.34</v>
+        <v>757.350399642613</v>
       </c>
       <c r="E8" s="8" t="n">
         <f aca="false">SUM(E4:E7)</f>
-        <v>457.05</v>
+        <v>457.034572318575</v>
       </c>
       <c r="F8" s="8" t="n">
         <f aca="false">SUM(F4:F7)</f>
-        <v>50.49</v>
+        <v>50.4890326755662</v>
       </c>
       <c r="G8" s="8" t="n">
         <f aca="false">SUM(G4:G7)</f>
-        <v>249.8</v>
+        <v>249.826794648472</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1207,7 +1205,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K103"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
@@ -1281,7 +1279,7 @@
       </c>
       <c r="E5" s="5" t="n">
         <f aca="false">SUM(F5:H5)</f>
-        <v>32.81</v>
+        <v>32.8148270267837</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>0</v>
@@ -1290,13 +1288,13 @@
         <v>0</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>32.81</v>
+        <v>32.8148270267837</v>
       </c>
       <c r="I5" s="4" t="n">
         <v>125</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>32.81</v>
+        <v>32.8148270267837</v>
       </c>
       <c r="K5" s="14" t="n">
         <v>0</v>
@@ -1317,22 +1315,22 @@
       </c>
       <c r="E6" s="5" t="n">
         <f aca="false">SUM(F6:H6)</f>
-        <v>29.9</v>
+        <v>29.9039484959109</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>8.95</v>
+        <v>8.94916596575711</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>20.95</v>
+        <v>20.9547825301538</v>
       </c>
       <c r="I6" s="4" t="n">
         <v>111</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>34.35</v>
+        <v>34.3465701717689</v>
       </c>
       <c r="K6" s="14" t="n">
         <v>0</v>
@@ -1353,7 +1351,7 @@
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">SUM(F7:H7)</f>
-        <v>25.54</v>
+        <v>25.5404328308278</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>0</v>
@@ -1362,13 +1360,13 @@
         <v>0</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>25.54</v>
+        <v>25.5404328308278</v>
       </c>
       <c r="I7" s="4" t="n">
         <v>108</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>29.84</v>
+        <v>29.8355663919971</v>
       </c>
       <c r="K7" s="14" t="n">
         <v>0</v>
@@ -1389,22 +1387,22 @@
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">SUM(F8:H8)</f>
-        <v>24.64</v>
+        <v>24.6311525361491</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>20.53</v>
+        <v>20.5254921809988</v>
       </c>
       <c r="G8" s="6" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>4.11</v>
+        <v>4.10566035515037</v>
       </c>
       <c r="I8" s="4" t="n">
         <v>101</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>24.63</v>
+        <v>24.6311525361491</v>
       </c>
       <c r="K8" s="15" t="n">
         <v>2</v>
@@ -1425,7 +1423,7 @@
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">SUM(F9:H9)</f>
-        <v>20.02</v>
+        <v>20.02434368</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>0</v>
@@ -1434,13 +1432,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>20.02</v>
+        <v>20.02434368</v>
       </c>
       <c r="I9" s="4" t="n">
         <v>186</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>20.02</v>
+        <v>20.02434368</v>
       </c>
       <c r="K9" s="14" t="n">
         <v>0</v>
@@ -1461,7 +1459,7 @@
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">SUM(F10:H10)</f>
-        <v>16.97</v>
+        <v>16.9689453224326</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>0</v>
@@ -1470,13 +1468,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>16.97</v>
+        <v>16.9689453224326</v>
       </c>
       <c r="I10" s="4" t="n">
         <v>111</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>16.97</v>
+        <v>16.9689453224326</v>
       </c>
       <c r="K10" s="15" t="n">
         <v>2.1</v>
@@ -1497,7 +1495,7 @@
       </c>
       <c r="E11" s="5" t="n">
         <f aca="false">SUM(F11:H11)</f>
-        <v>15.99</v>
+        <v>15.987</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>0</v>
@@ -1506,13 +1504,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>15.99</v>
+        <v>15.987</v>
       </c>
       <c r="I11" s="4" t="n">
         <v>125</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>15.99</v>
+        <v>15.987</v>
       </c>
       <c r="K11" s="14" t="n">
         <v>0</v>
@@ -1569,7 +1567,7 @@
       </c>
       <c r="E13" s="5" t="n">
         <f aca="false">SUM(F13:H13)</f>
-        <v>14.04</v>
+        <v>14.0415575471577</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>0</v>
@@ -1578,13 +1576,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>14.04</v>
+        <v>14.0415575471577</v>
       </c>
       <c r="I13" s="4" t="n">
         <v>124</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>14.04</v>
+        <v>14.0415575471577</v>
       </c>
       <c r="K13" s="14" t="n">
         <v>0</v>
@@ -1605,7 +1603,7 @@
       </c>
       <c r="E14" s="5" t="n">
         <f aca="false">SUM(F14:H14)</f>
-        <v>10.77</v>
+        <v>10.7731332766599</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>0</v>
@@ -1614,13 +1612,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="13" t="n">
-        <v>10.77</v>
+        <v>10.7731332766599</v>
       </c>
       <c r="I14" s="4" t="n">
         <v>96</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>20.34</v>
+        <v>20.3448108030086</v>
       </c>
       <c r="K14" s="14" t="n">
         <v>0</v>
@@ -1641,7 +1639,7 @@
       </c>
       <c r="E15" s="5" t="n">
         <f aca="false">SUM(F15:H15)</f>
-        <v>9.59</v>
+        <v>9.59333920000001</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>0</v>
@@ -1650,16 +1648,16 @@
         <v>0</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>9.59</v>
+        <v>9.59333920000001</v>
       </c>
       <c r="I15" s="4" t="n">
         <v>184</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>9.59</v>
+        <v>9.59333920000001</v>
       </c>
       <c r="K15" s="15" t="n">
-        <v>4.1</v>
+        <v>4.09999999999999</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1677,7 +1675,7 @@
       </c>
       <c r="E16" s="5" t="n">
         <f aca="false">SUM(F16:H16)</f>
-        <v>8.39</v>
+        <v>8.39289944188658</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>0</v>
@@ -1686,13 +1684,13 @@
         <v>0</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>8.39</v>
+        <v>8.39289944188658</v>
       </c>
       <c r="I16" s="4" t="n">
         <v>133</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>9.69</v>
+        <v>9.69094282016051</v>
       </c>
       <c r="K16" s="14" t="n">
         <v>0</v>
@@ -1713,7 +1711,7 @@
       </c>
       <c r="E17" s="5" t="n">
         <f aca="false">SUM(F17:H17)</f>
-        <v>6.79</v>
+        <v>6.791192096</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>0</v>
@@ -1722,13 +1720,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>6.79</v>
+        <v>6.791192096</v>
       </c>
       <c r="I17" s="4" t="n">
         <v>208</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>6.79</v>
+        <v>6.791192096</v>
       </c>
       <c r="K17" s="14" t="n">
         <v>0</v>
@@ -1749,7 +1747,7 @@
       </c>
       <c r="E18" s="5" t="n">
         <f aca="false">SUM(F18:H18)</f>
-        <v>6.12</v>
+        <v>6.11666481737043</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>0</v>
@@ -1758,13 +1756,13 @@
         <v>0</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>6.12</v>
+        <v>6.11666481737043</v>
       </c>
       <c r="I18" s="4" t="n">
         <v>128</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>6.12</v>
+        <v>6.11666481737043</v>
       </c>
       <c r="K18" s="14" t="n">
         <v>0</v>
@@ -1785,7 +1783,7 @@
       </c>
       <c r="E19" s="5" t="n">
         <f aca="false">SUM(F19:H19)</f>
-        <v>5.43</v>
+        <v>5.43362912409521</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>0</v>
@@ -1794,13 +1792,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>5.43</v>
+        <v>5.43362912409521</v>
       </c>
       <c r="I19" s="4" t="n">
         <v>120</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>5.43</v>
+        <v>5.43362912409521</v>
       </c>
       <c r="K19" s="14" t="n">
         <v>0</v>
@@ -1821,7 +1819,7 @@
       </c>
       <c r="E20" s="5" t="n">
         <f aca="false">SUM(F20:H20)</f>
-        <v>5.14</v>
+        <v>5.135805</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>0</v>
@@ -1830,13 +1828,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>5.14</v>
+        <v>5.135805</v>
       </c>
       <c r="I20" s="4" t="n">
         <v>182</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>5.14</v>
+        <v>5.135805</v>
       </c>
       <c r="K20" s="14" t="n">
         <v>0</v>
@@ -1857,7 +1855,7 @@
       </c>
       <c r="E21" s="5" t="n">
         <f aca="false">SUM(F21:H21)</f>
-        <v>3.78</v>
+        <v>3.7845792</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>0</v>
@@ -1866,13 +1864,13 @@
         <v>0</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>3.78</v>
+        <v>3.7845792</v>
       </c>
       <c r="I21" s="4" t="n">
         <v>138</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>3.78</v>
+        <v>3.7845792</v>
       </c>
       <c r="K21" s="14" t="n">
         <v>0</v>
@@ -1893,7 +1891,7 @@
       </c>
       <c r="E22" s="5" t="n">
         <f aca="false">SUM(F22:H22)</f>
-        <v>3.41</v>
+        <v>3.41136734497612</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>0</v>
@@ -1902,13 +1900,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>3.41</v>
+        <v>3.41136734497612</v>
       </c>
       <c r="I22" s="4" t="n">
         <v>110</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>3.41</v>
+        <v>3.41136734497612</v>
       </c>
       <c r="K22" s="14" t="n">
         <v>0</v>
@@ -1929,7 +1927,7 @@
       </c>
       <c r="E23" s="5" t="n">
         <f aca="false">SUM(F23:H23)</f>
-        <v>3.32</v>
+        <v>3.32262312468675</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>0</v>
@@ -1938,13 +1936,13 @@
         <v>0</v>
       </c>
       <c r="H23" s="13" t="n">
-        <v>3.32</v>
+        <v>3.32262312468675</v>
       </c>
       <c r="I23" s="4" t="n">
         <v>100</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>3.32</v>
+        <v>3.32262312468675</v>
       </c>
       <c r="K23" s="14" t="n">
         <v>0</v>
@@ -1965,7 +1963,7 @@
       </c>
       <c r="E24" s="5" t="n">
         <f aca="false">SUM(F24:H24)</f>
-        <v>2.87</v>
+        <v>2.87376537987296</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>0</v>
@@ -1974,13 +1972,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="13" t="n">
-        <v>2.87</v>
+        <v>2.87376537987296</v>
       </c>
       <c r="I24" s="4" t="n">
         <v>96</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>10.62</v>
+        <v>10.6181676337717</v>
       </c>
       <c r="K24" s="14" t="n">
         <v>0</v>
@@ -2001,7 +1999,7 @@
       </c>
       <c r="E25" s="5" t="n">
         <f aca="false">SUM(F25:H25)</f>
-        <v>2.46</v>
+        <v>2.4611925</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>0</v>
@@ -2010,13 +2008,13 @@
         <v>0</v>
       </c>
       <c r="H25" s="13" t="n">
-        <v>2.46</v>
+        <v>2.4611925</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>119</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>2.46</v>
+        <v>2.4611925</v>
       </c>
       <c r="K25" s="14" t="n">
         <v>0</v>
@@ -2037,7 +2035,7 @@
       </c>
       <c r="E26" s="5" t="n">
         <f aca="false">SUM(F26:H26)</f>
-        <v>2.43</v>
+        <v>2.431315</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>0</v>
@@ -2046,13 +2044,13 @@
         <v>0</v>
       </c>
       <c r="H26" s="13" t="n">
-        <v>2.43</v>
+        <v>2.431315</v>
       </c>
       <c r="I26" s="4" t="n">
         <v>112</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>3.45</v>
+        <v>3.4545625</v>
       </c>
       <c r="K26" s="14" t="n">
         <v>0</v>
@@ -2073,7 +2071,7 @@
       </c>
       <c r="E27" s="5" t="n">
         <f aca="false">SUM(F27:H27)</f>
-        <v>2.3</v>
+        <v>2.29685805039574</v>
       </c>
       <c r="F27" s="6" t="n">
         <v>0</v>
@@ -2082,13 +2080,13 @@
         <v>0</v>
       </c>
       <c r="H27" s="13" t="n">
-        <v>2.3</v>
+        <v>2.29685805039574</v>
       </c>
       <c r="I27" s="4" t="n">
         <v>116</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>5.4</v>
+        <v>5.40154390180969</v>
       </c>
       <c r="K27" s="14" t="n">
         <v>0</v>
@@ -2109,7 +2107,7 @@
       </c>
       <c r="E28" s="5" t="n">
         <f aca="false">SUM(F28:H28)</f>
-        <v>2.06</v>
+        <v>2.06041052800004</v>
       </c>
       <c r="F28" s="6" t="n">
         <v>0</v>
@@ -2118,13 +2116,13 @@
         <v>0</v>
       </c>
       <c r="H28" s="13" t="n">
-        <v>2.06</v>
+        <v>2.06041052800004</v>
       </c>
       <c r="I28" s="4" t="n">
         <v>111</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>2.06</v>
+        <v>2.06041052800004</v>
       </c>
       <c r="K28" s="14" t="n">
         <v>0</v>
@@ -2145,7 +2143,7 @@
       </c>
       <c r="E29" s="5" t="n">
         <f aca="false">SUM(F29:H29)</f>
-        <v>1.98</v>
+        <v>1.978658352</v>
       </c>
       <c r="F29" s="6" t="n">
         <v>0</v>
@@ -2154,13 +2152,13 @@
         <v>0</v>
       </c>
       <c r="H29" s="13" t="n">
-        <v>1.98</v>
+        <v>1.978658352</v>
       </c>
       <c r="I29" s="4" t="n">
         <v>208</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>1.98</v>
+        <v>1.978658352</v>
       </c>
       <c r="K29" s="14" t="n">
         <v>0</v>
@@ -2181,7 +2179,7 @@
       </c>
       <c r="E30" s="5" t="n">
         <f aca="false">SUM(F30:H30)</f>
-        <v>1.68</v>
+        <v>1.6796943760219</v>
       </c>
       <c r="F30" s="6" t="n">
         <v>0</v>
@@ -2190,13 +2188,13 @@
         <v>0</v>
       </c>
       <c r="H30" s="13" t="n">
-        <v>1.68</v>
+        <v>1.6796943760219</v>
       </c>
       <c r="I30" s="4" t="n">
         <v>94</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>1.68</v>
+        <v>1.6796943760219</v>
       </c>
       <c r="K30" s="15" t="n">
         <v>4.3</v>
@@ -2217,7 +2215,7 @@
       </c>
       <c r="E31" s="5" t="n">
         <f aca="false">SUM(F31:H31)</f>
-        <v>1.67</v>
+        <v>1.66718272</v>
       </c>
       <c r="F31" s="6" t="n">
         <v>0</v>
@@ -2226,13 +2224,13 @@
         <v>0</v>
       </c>
       <c r="H31" s="13" t="n">
-        <v>1.67</v>
+        <v>1.66718272</v>
       </c>
       <c r="I31" s="4" t="n">
         <v>163</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>1.67</v>
+        <v>1.66718272</v>
       </c>
       <c r="K31" s="14" t="n">
         <v>0</v>
@@ -2253,7 +2251,7 @@
       </c>
       <c r="E32" s="5" t="n">
         <f aca="false">SUM(F32:H32)</f>
-        <v>1.49</v>
+        <v>1.49284396800001</v>
       </c>
       <c r="F32" s="6" t="n">
         <v>0</v>
@@ -2262,13 +2260,13 @@
         <v>0</v>
       </c>
       <c r="H32" s="13" t="n">
-        <v>1.49</v>
+        <v>1.49284396800001</v>
       </c>
       <c r="I32" s="4" t="n">
         <v>159</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>1.49</v>
+        <v>1.49284396800001</v>
       </c>
       <c r="K32" s="14" t="n">
         <v>0</v>
@@ -2289,7 +2287,7 @@
       </c>
       <c r="E33" s="5" t="n">
         <f aca="false">SUM(F33:H33)</f>
-        <v>1.05</v>
+        <v>1.050544896</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
@@ -2298,13 +2296,13 @@
         <v>0</v>
       </c>
       <c r="H33" s="13" t="n">
-        <v>1.05</v>
+        <v>1.050544896</v>
       </c>
       <c r="I33" s="4" t="n">
         <v>139</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>12.39</v>
+        <v>12.385894656</v>
       </c>
       <c r="K33" s="14" t="n">
         <v>0</v>
@@ -2325,7 +2323,7 @@
       </c>
       <c r="E34" s="5" t="n">
         <f aca="false">SUM(F34:H34)</f>
-        <v>0.81</v>
+        <v>0.810000000000002</v>
       </c>
       <c r="F34" s="6" t="n">
         <v>0</v>
@@ -2334,13 +2332,13 @@
         <v>0</v>
       </c>
       <c r="H34" s="13" t="n">
-        <v>0.81</v>
+        <v>0.810000000000002</v>
       </c>
       <c r="I34" s="4" t="n">
         <v>118</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>0.81</v>
+        <v>0.810000000000002</v>
       </c>
       <c r="K34" s="14" t="n">
         <v>0</v>
@@ -2361,7 +2359,7 @@
       </c>
       <c r="E35" s="5" t="n">
         <f aca="false">SUM(F35:H35)</f>
-        <v>0.36</v>
+        <v>0.364999999999998</v>
       </c>
       <c r="F35" s="6" t="n">
         <v>0</v>
@@ -2370,13 +2368,13 @@
         <v>0</v>
       </c>
       <c r="H35" s="13" t="n">
-        <v>0.36</v>
+        <v>0.364999999999998</v>
       </c>
       <c r="I35" s="4" t="n">
         <v>118</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>0.36</v>
+        <v>0.364999999999998</v>
       </c>
       <c r="K35" s="14" t="n">
         <v>0</v>
@@ -2397,7 +2395,7 @@
       </c>
       <c r="E36" s="5" t="n">
         <f aca="false">SUM(F36:H36)</f>
-        <v>0.18</v>
+        <v>0.17734696</v>
       </c>
       <c r="F36" s="6" t="n">
         <v>0</v>
@@ -2406,13 +2404,13 @@
         <v>0</v>
       </c>
       <c r="H36" s="13" t="n">
-        <v>0.18</v>
+        <v>0.17734696</v>
       </c>
       <c r="I36" s="4" t="n">
         <v>138</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0.18</v>
+        <v>0.17734696</v>
       </c>
       <c r="K36" s="14" t="n">
         <v>0</v>
@@ -2433,7 +2431,7 @@
       </c>
       <c r="E37" s="5" t="n">
         <f aca="false">SUM(F37:H37)</f>
-        <v>0.06</v>
+        <v>0.0619999999999976</v>
       </c>
       <c r="F37" s="6" t="n">
         <v>0</v>
@@ -2442,13 +2440,13 @@
         <v>0</v>
       </c>
       <c r="H37" s="13" t="n">
-        <v>0.06</v>
+        <v>0.0619999999999976</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>124</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>0.06</v>
+        <v>0.0619999999999976</v>
       </c>
       <c r="K37" s="14" t="n">
         <v>0</v>
@@ -2469,7 +2467,7 @@
       </c>
       <c r="E38" s="5" t="n">
         <f aca="false">SUM(F38:H38)</f>
-        <v>0.02</v>
+        <v>0.0172000000000008</v>
       </c>
       <c r="F38" s="6" t="n">
         <v>0</v>
@@ -2478,13 +2476,13 @@
         <v>0</v>
       </c>
       <c r="H38" s="13" t="n">
-        <v>0.02</v>
+        <v>0.0172000000000008</v>
       </c>
       <c r="I38" s="4" t="n">
         <v>120</v>
       </c>
       <c r="J38" s="6" t="n">
-        <v>0.02</v>
+        <v>0.0172000000000008</v>
       </c>
       <c r="K38" s="14" t="n">
         <v>0</v>
@@ -2505,13 +2503,13 @@
       </c>
       <c r="E39" s="5" t="n">
         <f aca="false">SUM(F39:H39)</f>
-        <v>21.38</v>
+        <v>21.377012416</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>15.58</v>
+        <v>15.579142656</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>5.8</v>
+        <v>5.79786976000001</v>
       </c>
       <c r="H39" s="6" t="n">
         <v>0</v>
@@ -2520,7 +2518,7 @@
         <v>67</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>21.38</v>
+        <v>21.377012416</v>
       </c>
       <c r="K39" s="14" t="n">
         <v>0</v>
@@ -2541,13 +2539,13 @@
       </c>
       <c r="E40" s="5" t="n">
         <f aca="false">SUM(F40:H40)</f>
-        <v>9.05</v>
+        <v>9.04905037447167</v>
       </c>
       <c r="F40" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>9.05</v>
+        <v>9.04905037447167</v>
       </c>
       <c r="H40" s="6" t="n">
         <v>0</v>
@@ -2556,7 +2554,7 @@
         <v>65</v>
       </c>
       <c r="J40" s="6" t="n">
-        <v>9.05</v>
+        <v>9.04905037447167</v>
       </c>
       <c r="K40" s="15" t="n">
         <v>4.05</v>
@@ -2577,13 +2575,13 @@
       </c>
       <c r="E41" s="5" t="n">
         <f aca="false">SUM(F41:H41)</f>
-        <v>7.39</v>
+        <v>7.39196666203888</v>
       </c>
       <c r="F41" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="6" t="n">
-        <v>7.39</v>
+        <v>7.39196666203888</v>
       </c>
       <c r="H41" s="6" t="n">
         <v>0</v>
@@ -2592,10 +2590,10 @@
         <v>68</v>
       </c>
       <c r="J41" s="6" t="n">
-        <v>7.39</v>
+        <v>7.39196666203888</v>
       </c>
       <c r="K41" s="15" t="n">
-        <v>1.95</v>
+        <v>1.94999999999999</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2628,7 +2626,7 @@
         <v>88</v>
       </c>
       <c r="J42" s="6" t="n">
-        <v>9.95</v>
+        <v>9.9489</v>
       </c>
       <c r="K42" s="14" t="n">
         <v>0</v>
@@ -2649,13 +2647,13 @@
       </c>
       <c r="E43" s="5" t="n">
         <f aca="false">SUM(F43:H43)</f>
-        <v>4.91</v>
+        <v>4.91416944529855</v>
       </c>
       <c r="F43" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G43" s="6" t="n">
-        <v>4.91</v>
+        <v>4.91416944529855</v>
       </c>
       <c r="H43" s="6" t="n">
         <v>0</v>
@@ -2664,7 +2662,7 @@
         <v>65</v>
       </c>
       <c r="J43" s="6" t="n">
-        <v>4.91</v>
+        <v>4.91416944529855</v>
       </c>
       <c r="K43" s="14" t="n">
         <v>0</v>
@@ -2685,13 +2683,13 @@
       </c>
       <c r="E44" s="5" t="n">
         <f aca="false">SUM(F44:H44)</f>
-        <v>4.39</v>
+        <v>4.38852000000001</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>2.39</v>
+        <v>2.390325</v>
       </c>
       <c r="G44" s="6" t="n">
-        <v>2</v>
+        <v>1.99819500000001</v>
       </c>
       <c r="H44" s="6" t="n">
         <v>0</v>
@@ -2700,7 +2698,7 @@
         <v>70</v>
       </c>
       <c r="J44" s="6" t="n">
-        <v>4.39</v>
+        <v>4.38852000000001</v>
       </c>
       <c r="K44" s="14" t="n">
         <v>0</v>
@@ -2721,13 +2719,13 @@
       </c>
       <c r="E45" s="5" t="n">
         <f aca="false">SUM(F45:H45)</f>
-        <v>3.09</v>
+        <v>3.09150749999996</v>
       </c>
       <c r="F45" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G45" s="6" t="n">
-        <v>3.09</v>
+        <v>3.09150749999996</v>
       </c>
       <c r="H45" s="6" t="n">
         <v>0</v>
@@ -2736,7 +2734,7 @@
         <v>66</v>
       </c>
       <c r="J45" s="6" t="n">
-        <v>3.09</v>
+        <v>3.09150749999996</v>
       </c>
       <c r="K45" s="14" t="n">
         <v>0</v>
@@ -2757,13 +2755,13 @@
       </c>
       <c r="E46" s="5" t="n">
         <f aca="false">SUM(F46:H46)</f>
-        <v>2.13</v>
+        <v>2.1282</v>
       </c>
       <c r="F46" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G46" s="6" t="n">
-        <v>2.13</v>
+        <v>2.1282</v>
       </c>
       <c r="H46" s="6" t="n">
         <v>0</v>
@@ -2772,7 +2770,7 @@
         <v>88</v>
       </c>
       <c r="J46" s="6" t="n">
-        <v>21.9</v>
+        <v>21.8961</v>
       </c>
       <c r="K46" s="14" t="n">
         <v>0</v>
@@ -2793,13 +2791,13 @@
       </c>
       <c r="E47" s="5" t="n">
         <f aca="false">SUM(F47:H47)</f>
-        <v>0.4</v>
+        <v>0.398907968</v>
       </c>
       <c r="F47" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G47" s="6" t="n">
-        <v>0.4</v>
+        <v>0.398907968</v>
       </c>
       <c r="H47" s="6" t="n">
         <v>0</v>
@@ -2808,7 +2806,7 @@
         <v>68</v>
       </c>
       <c r="J47" s="6" t="n">
-        <v>0.4</v>
+        <v>0.398907968</v>
       </c>
       <c r="K47" s="14" t="n">
         <v>0</v>
@@ -2829,10 +2827,10 @@
       </c>
       <c r="E48" s="5" t="n">
         <f aca="false">SUM(F48:H48)</f>
-        <v>23.92</v>
+        <v>23.918199616</v>
       </c>
       <c r="F48" s="6" t="n">
-        <v>23.92</v>
+        <v>23.918199616</v>
       </c>
       <c r="G48" s="6" t="n">
         <v>0</v>
@@ -2844,10 +2842,10 @@
         <v>47</v>
       </c>
       <c r="J48" s="6" t="n">
-        <v>23.92</v>
+        <v>23.918199616</v>
       </c>
       <c r="K48" s="15" t="n">
-        <v>7.05</v>
+        <v>7.05000000000001</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2865,10 +2863,10 @@
       </c>
       <c r="E49" s="5" t="n">
         <f aca="false">SUM(F49:H49)</f>
-        <v>15.1</v>
+        <v>15.1022607216639</v>
       </c>
       <c r="F49" s="6" t="n">
-        <v>15.1</v>
+        <v>15.1022607216639</v>
       </c>
       <c r="G49" s="6" t="n">
         <v>0</v>
@@ -2880,7 +2878,7 @@
         <v>42</v>
       </c>
       <c r="J49" s="6" t="n">
-        <v>15.1</v>
+        <v>15.1022607216639</v>
       </c>
       <c r="K49" s="15" t="n">
         <v>4.13</v>
@@ -2901,10 +2899,10 @@
       </c>
       <c r="E50" s="5" t="n">
         <f aca="false">SUM(F50:H50)</f>
-        <v>14.86</v>
+        <v>14.8571984059727</v>
       </c>
       <c r="F50" s="6" t="n">
-        <v>14.86</v>
+        <v>14.8571984059727</v>
       </c>
       <c r="G50" s="6" t="n">
         <v>0</v>
@@ -2916,7 +2914,7 @@
         <v>37</v>
       </c>
       <c r="J50" s="6" t="n">
-        <v>14.86</v>
+        <v>14.8571984059727</v>
       </c>
       <c r="K50" s="18" t="s">
         <v>76</v>
@@ -2937,10 +2935,10 @@
       </c>
       <c r="E51" s="5" t="n">
         <f aca="false">SUM(F51:H51)</f>
-        <v>13.01</v>
+        <v>13.0084675</v>
       </c>
       <c r="F51" s="6" t="n">
-        <v>13.01</v>
+        <v>13.0084675</v>
       </c>
       <c r="G51" s="6" t="n">
         <v>0</v>
@@ -2952,7 +2950,7 @@
         <v>45</v>
       </c>
       <c r="J51" s="6" t="n">
-        <v>13.01</v>
+        <v>13.0084675</v>
       </c>
       <c r="K51" s="14" t="n">
         <v>0</v>
@@ -2973,10 +2971,10 @@
       </c>
       <c r="E52" s="5" t="n">
         <f aca="false">SUM(F52:H52)</f>
-        <v>9.88</v>
+        <v>9.8822976</v>
       </c>
       <c r="F52" s="6" t="n">
-        <v>9.88</v>
+        <v>9.8822976</v>
       </c>
       <c r="G52" s="6" t="n">
         <v>0</v>
@@ -2988,7 +2986,7 @@
         <v>32</v>
       </c>
       <c r="J52" s="6" t="n">
-        <v>9.88</v>
+        <v>9.8822976</v>
       </c>
       <c r="K52" s="18" t="s">
         <v>76</v>
@@ -3009,10 +3007,10 @@
       </c>
       <c r="E53" s="5" t="n">
         <f aca="false">SUM(F53:H53)</f>
-        <v>9.48</v>
+        <v>9.48384355438487</v>
       </c>
       <c r="F53" s="6" t="n">
-        <v>9.48</v>
+        <v>9.48384355438487</v>
       </c>
       <c r="G53" s="6" t="n">
         <v>0</v>
@@ -3024,7 +3022,7 @@
         <v>42</v>
       </c>
       <c r="J53" s="6" t="n">
-        <v>9.48</v>
+        <v>9.48384355438487</v>
       </c>
       <c r="K53" s="14" t="n">
         <v>0</v>
@@ -3045,10 +3043,10 @@
       </c>
       <c r="E54" s="5" t="n">
         <f aca="false">SUM(F54:H54)</f>
-        <v>9.18</v>
+        <v>9.17650559999998</v>
       </c>
       <c r="F54" s="6" t="n">
-        <v>9.18</v>
+        <v>9.17650559999998</v>
       </c>
       <c r="G54" s="6" t="n">
         <v>0</v>
@@ -3060,7 +3058,7 @@
         <v>32</v>
       </c>
       <c r="J54" s="6" t="n">
-        <v>47.86</v>
+        <v>47.8587936</v>
       </c>
       <c r="K54" s="18" t="s">
         <v>76</v>
@@ -3081,10 +3079,10 @@
       </c>
       <c r="E55" s="5" t="n">
         <f aca="false">SUM(F55:H55)</f>
-        <v>8.83</v>
+        <v>8.8327184</v>
       </c>
       <c r="F55" s="6" t="n">
-        <v>8.83</v>
+        <v>8.8327184</v>
       </c>
       <c r="G55" s="6" t="n">
         <v>0</v>
@@ -3096,7 +3094,7 @@
         <v>34</v>
       </c>
       <c r="J55" s="6" t="n">
-        <v>8.83</v>
+        <v>8.8327184</v>
       </c>
       <c r="K55" s="18" t="s">
         <v>76</v>
@@ -3117,10 +3115,10 @@
       </c>
       <c r="E56" s="5" t="n">
         <f aca="false">SUM(F56:H56)</f>
-        <v>7.16</v>
+        <v>7.15569465599997</v>
       </c>
       <c r="F56" s="6" t="n">
-        <v>7.16</v>
+        <v>7.15569465599997</v>
       </c>
       <c r="G56" s="6" t="n">
         <v>0</v>
@@ -3132,7 +3130,7 @@
         <v>44</v>
       </c>
       <c r="J56" s="6" t="n">
-        <v>7.16</v>
+        <v>7.15569465599997</v>
       </c>
       <c r="K56" s="14" t="n">
         <v>0</v>
@@ -3153,10 +3151,10 @@
       </c>
       <c r="E57" s="5" t="n">
         <f aca="false">SUM(F57:H57)</f>
-        <v>6.79</v>
+        <v>6.78931658298102</v>
       </c>
       <c r="F57" s="6" t="n">
-        <v>6.79</v>
+        <v>6.78931658298102</v>
       </c>
       <c r="G57" s="6" t="n">
         <v>0</v>
@@ -3168,10 +3166,10 @@
         <v>38</v>
       </c>
       <c r="J57" s="6" t="n">
-        <v>14.62</v>
+        <v>14.6224114638618</v>
       </c>
       <c r="K57" s="15" t="n">
-        <v>4.15</v>
+        <v>4.15000000000001</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3189,10 +3187,10 @@
       </c>
       <c r="E58" s="5" t="n">
         <f aca="false">SUM(F58:H58)</f>
-        <v>5.89</v>
+        <v>5.8923136</v>
       </c>
       <c r="F58" s="6" t="n">
-        <v>5.89</v>
+        <v>5.8923136</v>
       </c>
       <c r="G58" s="6" t="n">
         <v>0</v>
@@ -3204,7 +3202,7 @@
         <v>33</v>
       </c>
       <c r="J58" s="6" t="n">
-        <v>5.89</v>
+        <v>5.8923136</v>
       </c>
       <c r="K58" s="18" t="s">
         <v>76</v>
@@ -3225,10 +3223,10 @@
       </c>
       <c r="E59" s="5" t="n">
         <f aca="false">SUM(F59:H59)</f>
-        <v>4.89</v>
+        <v>4.8935464</v>
       </c>
       <c r="F59" s="6" t="n">
-        <v>4.89</v>
+        <v>4.8935464</v>
       </c>
       <c r="G59" s="6" t="n">
         <v>0</v>
@@ -3240,7 +3238,7 @@
         <v>34</v>
       </c>
       <c r="J59" s="6" t="n">
-        <v>21.68</v>
+        <v>21.6809284</v>
       </c>
       <c r="K59" s="18" t="s">
         <v>76</v>
@@ -3261,10 +3259,10 @@
       </c>
       <c r="E60" s="5" t="n">
         <f aca="false">SUM(F60:H60)</f>
-        <v>4.63</v>
+        <v>4.63078547616842</v>
       </c>
       <c r="F60" s="6" t="n">
-        <v>4.63</v>
+        <v>4.63078547616842</v>
       </c>
       <c r="G60" s="6" t="n">
         <v>0</v>
@@ -3276,7 +3274,7 @@
         <v>49</v>
       </c>
       <c r="J60" s="6" t="n">
-        <v>4.63</v>
+        <v>4.63078547616842</v>
       </c>
       <c r="K60" s="14" t="n">
         <v>0</v>
@@ -3297,10 +3295,10 @@
       </c>
       <c r="E61" s="5" t="n">
         <f aca="false">SUM(F61:H61)</f>
-        <v>3.48</v>
+        <v>3.47849600000004</v>
       </c>
       <c r="F61" s="6" t="n">
-        <v>3.48</v>
+        <v>3.47849600000004</v>
       </c>
       <c r="G61" s="6" t="n">
         <v>0</v>
@@ -3312,7 +3310,7 @@
         <v>33</v>
       </c>
       <c r="J61" s="6" t="n">
-        <v>49</v>
+        <v>49.0019648</v>
       </c>
       <c r="K61" s="18" t="s">
         <v>76</v>
@@ -3333,10 +3331,10 @@
       </c>
       <c r="E62" s="5" t="n">
         <f aca="false">SUM(F62:H62)</f>
-        <v>3.03</v>
+        <v>3.03031600000002</v>
       </c>
       <c r="F62" s="6" t="n">
-        <v>3.03</v>
+        <v>3.03031600000002</v>
       </c>
       <c r="G62" s="6" t="n">
         <v>0</v>
@@ -3348,7 +3346,7 @@
         <v>37</v>
       </c>
       <c r="J62" s="6" t="n">
-        <v>3.03</v>
+        <v>3.03031600000002</v>
       </c>
       <c r="K62" s="18" t="s">
         <v>76</v>
@@ -3369,10 +3367,10 @@
       </c>
       <c r="E63" s="5" t="n">
         <f aca="false">SUM(F63:H63)</f>
-        <v>2.92</v>
+        <v>2.91910249999999</v>
       </c>
       <c r="F63" s="6" t="n">
-        <v>2.92</v>
+        <v>2.91910249999999</v>
       </c>
       <c r="G63" s="6" t="n">
         <v>0</v>
@@ -3384,7 +3382,7 @@
         <v>47</v>
       </c>
       <c r="J63" s="6" t="n">
-        <v>2.92</v>
+        <v>2.91910249999999</v>
       </c>
       <c r="K63" s="14" t="n">
         <v>0</v>
@@ -3405,10 +3403,10 @@
       </c>
       <c r="E64" s="5" t="n">
         <f aca="false">SUM(F64:H64)</f>
-        <v>2.58</v>
+        <v>2.58205749999999</v>
       </c>
       <c r="F64" s="6" t="n">
-        <v>2.58</v>
+        <v>2.58205749999999</v>
       </c>
       <c r="G64" s="6" t="n">
         <v>0</v>
@@ -3420,7 +3418,7 @@
         <v>44</v>
       </c>
       <c r="J64" s="6" t="n">
-        <v>5.29</v>
+        <v>5.29030749999999</v>
       </c>
       <c r="K64" s="14" t="n">
         <v>0</v>
@@ -3441,10 +3439,10 @@
       </c>
       <c r="E65" s="5" t="n">
         <f aca="false">SUM(F65:H65)</f>
-        <v>2.4</v>
+        <v>2.40446237338101</v>
       </c>
       <c r="F65" s="6" t="n">
-        <v>2.4</v>
+        <v>2.40446237338101</v>
       </c>
       <c r="G65" s="6" t="n">
         <v>0</v>
@@ -3456,7 +3454,7 @@
         <v>58</v>
       </c>
       <c r="J65" s="6" t="n">
-        <v>33.52</v>
+        <v>33.5239322420628</v>
       </c>
       <c r="K65" s="14" t="n">
         <v>0</v>
@@ -3477,10 +3475,10 @@
       </c>
       <c r="E66" s="5" t="n">
         <f aca="false">SUM(F66:H66)</f>
-        <v>1.35</v>
+        <v>1.35044088702466</v>
       </c>
       <c r="F66" s="6" t="n">
-        <v>1.35</v>
+        <v>1.35044088702466</v>
       </c>
       <c r="G66" s="6" t="n">
         <v>0</v>
@@ -3492,7 +3490,7 @@
         <v>49</v>
       </c>
       <c r="J66" s="6" t="n">
-        <v>1.35</v>
+        <v>1.35044088702466</v>
       </c>
       <c r="K66" s="14" t="n">
         <v>0</v>
@@ -3513,10 +3511,10 @@
       </c>
       <c r="E67" s="5" t="n">
         <f aca="false">SUM(F67:H67)</f>
-        <v>0.02</v>
+        <v>0.0195334399999876</v>
       </c>
       <c r="F67" s="6" t="n">
-        <v>0.02</v>
+        <v>0.0195334399999876</v>
       </c>
       <c r="G67" s="6" t="n">
         <v>0</v>
@@ -3528,7 +3526,7 @@
         <v>53</v>
       </c>
       <c r="J67" s="6" t="n">
-        <v>0.02</v>
+        <v>0.0195334399999876</v>
       </c>
       <c r="K67" s="14" t="n">
         <v>0</v>
@@ -3549,10 +3547,10 @@
       </c>
       <c r="E68" s="5" t="n">
         <f aca="false">SUM(F68:H68)</f>
-        <v>56.23</v>
+        <v>56.233144</v>
       </c>
       <c r="F68" s="6" t="n">
-        <v>56.23</v>
+        <v>56.233144</v>
       </c>
       <c r="G68" s="6" t="n">
         <v>0</v>
@@ -3564,10 +3562,10 @@
         <v>41</v>
       </c>
       <c r="J68" s="6" t="n">
-        <v>91.13</v>
+        <v>91.1346208</v>
       </c>
       <c r="K68" s="15" t="n">
-        <v>8.02</v>
+        <v>8.02399999999999</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3585,10 +3583,10 @@
       </c>
       <c r="E69" s="5" t="n">
         <f aca="false">SUM(F69:H69)</f>
-        <v>44.64</v>
+        <v>44.6432888</v>
       </c>
       <c r="F69" s="6" t="n">
-        <v>44.64</v>
+        <v>44.6432888</v>
       </c>
       <c r="G69" s="6" t="n">
         <v>0</v>
@@ -3600,10 +3598,10 @@
         <v>45</v>
       </c>
       <c r="J69" s="6" t="n">
-        <v>44.64</v>
+        <v>44.6432888</v>
       </c>
       <c r="K69" s="15" t="n">
-        <v>4.91</v>
+        <v>4.912</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3621,10 +3619,10 @@
       </c>
       <c r="E70" s="5" t="n">
         <f aca="false">SUM(F70:H70)</f>
-        <v>27.43</v>
+        <v>27.4279504</v>
       </c>
       <c r="F70" s="6" t="n">
-        <v>27.43</v>
+        <v>27.4279504</v>
       </c>
       <c r="G70" s="6" t="n">
         <v>0</v>
@@ -3636,7 +3634,7 @@
         <v>50</v>
       </c>
       <c r="J70" s="6" t="n">
-        <v>27.43</v>
+        <v>27.4279504</v>
       </c>
       <c r="K70" s="14" t="n">
         <v>0</v>
@@ -3657,10 +3655,10 @@
       </c>
       <c r="E71" s="5" t="n">
         <f aca="false">SUM(F71:H71)</f>
-        <v>16.8</v>
+        <v>16.7964288</v>
       </c>
       <c r="F71" s="6" t="n">
-        <v>16.8</v>
+        <v>16.7964288</v>
       </c>
       <c r="G71" s="6" t="n">
         <v>0</v>
@@ -3672,10 +3670,10 @@
         <v>52</v>
       </c>
       <c r="J71" s="6" t="n">
-        <v>58.72</v>
+        <v>58.720704</v>
       </c>
       <c r="K71" s="15" t="n">
-        <v>17.53</v>
+        <v>17.527</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3693,10 +3691,10 @@
       </c>
       <c r="E72" s="5" t="n">
         <f aca="false">SUM(F72:H72)</f>
-        <v>11.12</v>
+        <v>11.123178688</v>
       </c>
       <c r="F72" s="6" t="n">
-        <v>11.12</v>
+        <v>11.123178688</v>
       </c>
       <c r="G72" s="6" t="n">
         <v>0</v>
@@ -3708,7 +3706,7 @@
         <v>33</v>
       </c>
       <c r="J72" s="6" t="n">
-        <v>11.12</v>
+        <v>11.123178688</v>
       </c>
       <c r="K72" s="18" t="s">
         <v>76</v>
@@ -3729,10 +3727,10 @@
       </c>
       <c r="E73" s="5" t="n">
         <f aca="false">SUM(F73:H73)</f>
-        <v>0.63</v>
+        <v>0.634543680000022</v>
       </c>
       <c r="F73" s="6" t="n">
-        <v>0.63</v>
+        <v>0.634543680000022</v>
       </c>
       <c r="G73" s="6" t="n">
         <v>0</v>
@@ -3744,7 +3742,7 @@
         <v>38</v>
       </c>
       <c r="J73" s="6" t="n">
-        <v>62.64</v>
+        <v>62.6361697920001</v>
       </c>
       <c r="K73" s="14" t="n">
         <v>0</v>
@@ -3765,10 +3763,10 @@
       </c>
       <c r="E74" s="5" t="n">
         <f aca="false">SUM(F74:H74)</f>
-        <v>9.37</v>
+        <v>9.369212</v>
       </c>
       <c r="F74" s="6" t="n">
-        <v>9.37</v>
+        <v>9.369212</v>
       </c>
       <c r="G74" s="6" t="n">
         <v>0</v>
@@ -3780,7 +3778,7 @@
         <v>31</v>
       </c>
       <c r="J74" s="6" t="n">
-        <v>9.37</v>
+        <v>9.369212</v>
       </c>
       <c r="K74" s="18" t="s">
         <v>76</v>
@@ -3801,10 +3799,10 @@
       </c>
       <c r="E75" s="5" t="n">
         <f aca="false">SUM(F75:H75)</f>
-        <v>6.8</v>
+        <v>6.795064</v>
       </c>
       <c r="F75" s="6" t="n">
-        <v>6.8</v>
+        <v>6.795064</v>
       </c>
       <c r="G75" s="6" t="n">
         <v>0</v>
@@ -3816,7 +3814,7 @@
         <v>31</v>
       </c>
       <c r="J75" s="6" t="n">
-        <v>6.8</v>
+        <v>6.795064</v>
       </c>
       <c r="K75" s="18" t="s">
         <v>76</v>
@@ -3837,10 +3835,10 @@
       </c>
       <c r="E76" s="5" t="n">
         <f aca="false">SUM(F76:H76)</f>
-        <v>5.47</v>
+        <v>5.467136</v>
       </c>
       <c r="F76" s="6" t="n">
-        <v>5.47</v>
+        <v>5.467136</v>
       </c>
       <c r="G76" s="6" t="n">
         <v>0</v>
@@ -3852,7 +3850,7 @@
         <v>35</v>
       </c>
       <c r="J76" s="6" t="n">
-        <v>5.47</v>
+        <v>5.467136</v>
       </c>
       <c r="K76" s="18" t="s">
         <v>76</v>
@@ -3873,10 +3871,10 @@
       </c>
       <c r="E77" s="5" t="n">
         <f aca="false">SUM(F77:H77)</f>
-        <v>4.58</v>
+        <v>4.5791184</v>
       </c>
       <c r="F77" s="6" t="n">
-        <v>4.58</v>
+        <v>4.5791184</v>
       </c>
       <c r="G77" s="6" t="n">
         <v>0</v>
@@ -3888,7 +3886,7 @@
         <v>32</v>
       </c>
       <c r="J77" s="6" t="n">
-        <v>4.58</v>
+        <v>4.5791184</v>
       </c>
       <c r="K77" s="18" t="s">
         <v>76</v>
@@ -3909,10 +3907,10 @@
       </c>
       <c r="E78" s="5" t="n">
         <f aca="false">SUM(F78:H78)</f>
-        <v>4.49</v>
+        <v>4.494248</v>
       </c>
       <c r="F78" s="6" t="n">
-        <v>4.49</v>
+        <v>4.494248</v>
       </c>
       <c r="G78" s="6" t="n">
         <v>0</v>
@@ -3924,7 +3922,7 @@
         <v>60</v>
       </c>
       <c r="J78" s="6" t="n">
-        <v>4.49</v>
+        <v>4.494248</v>
       </c>
       <c r="K78" s="14" t="n">
         <v>0</v>
@@ -3945,10 +3943,10 @@
       </c>
       <c r="E79" s="5" t="n">
         <f aca="false">SUM(F79:H79)</f>
-        <v>3.98</v>
+        <v>3.9753</v>
       </c>
       <c r="F79" s="6" t="n">
-        <v>3.98</v>
+        <v>3.9753</v>
       </c>
       <c r="G79" s="6" t="n">
         <v>0</v>
@@ -3960,7 +3958,7 @@
         <v>34</v>
       </c>
       <c r="J79" s="6" t="n">
-        <v>3.98</v>
+        <v>3.9753</v>
       </c>
       <c r="K79" s="18" t="s">
         <v>76</v>
@@ -3981,10 +3979,10 @@
       </c>
       <c r="E80" s="5" t="n">
         <f aca="false">SUM(F80:H80)</f>
-        <v>1.04</v>
+        <v>1.0383108</v>
       </c>
       <c r="F80" s="6" t="n">
-        <v>1.04</v>
+        <v>1.0383108</v>
       </c>
       <c r="G80" s="6" t="n">
         <v>0</v>
@@ -3996,7 +3994,7 @@
         <v>33</v>
       </c>
       <c r="J80" s="6" t="n">
-        <v>1.04</v>
+        <v>1.0383108</v>
       </c>
       <c r="K80" s="18" t="s">
         <v>76</v>
@@ -4017,10 +4015,10 @@
       </c>
       <c r="E81" s="5" t="n">
         <f aca="false">SUM(F81:H81)</f>
-        <v>0.72</v>
+        <v>0.722176000000005</v>
       </c>
       <c r="F81" s="6" t="n">
-        <v>0.72</v>
+        <v>0.722176000000005</v>
       </c>
       <c r="G81" s="6" t="n">
         <v>0</v>
@@ -4032,7 +4030,7 @@
         <v>32</v>
       </c>
       <c r="J81" s="6" t="n">
-        <v>0.72</v>
+        <v>0.722176000000005</v>
       </c>
       <c r="K81" s="18" t="s">
         <v>76</v>
@@ -4053,10 +4051,10 @@
       </c>
       <c r="E82" s="5" t="n">
         <f aca="false">SUM(F82:H82)</f>
-        <v>0.11</v>
+        <v>0.111864</v>
       </c>
       <c r="F82" s="6" t="n">
-        <v>0.11</v>
+        <v>0.111864</v>
       </c>
       <c r="G82" s="6" t="n">
         <v>0</v>
@@ -4068,7 +4066,7 @@
         <v>37</v>
       </c>
       <c r="J82" s="6" t="n">
-        <v>0.11</v>
+        <v>0.111864</v>
       </c>
       <c r="K82" s="18" t="s">
         <v>76</v>
@@ -4089,10 +4087,10 @@
       </c>
       <c r="E83" s="5" t="n">
         <f aca="false">SUM(F83:H83)</f>
-        <v>0.09</v>
+        <v>0.0868599999999997</v>
       </c>
       <c r="F83" s="6" t="n">
-        <v>0.09</v>
+        <v>0.0868599999999997</v>
       </c>
       <c r="G83" s="6" t="n">
         <v>0</v>
@@ -4104,7 +4102,7 @@
         <v>37</v>
       </c>
       <c r="J83" s="6" t="n">
-        <v>0.09</v>
+        <v>0.0868599999999997</v>
       </c>
       <c r="K83" s="18" t="s">
         <v>76</v>
@@ -4125,10 +4123,10 @@
       </c>
       <c r="E84" s="5" t="n">
         <f aca="false">SUM(F84:H84)</f>
-        <v>0.03</v>
+        <v>0.026099999999996</v>
       </c>
       <c r="F84" s="6" t="n">
-        <v>0.03</v>
+        <v>0.026099999999996</v>
       </c>
       <c r="G84" s="6" t="n">
         <v>0</v>
@@ -4140,7 +4138,7 @@
         <v>57</v>
       </c>
       <c r="J84" s="6" t="n">
-        <v>0.03</v>
+        <v>0.026099999999996</v>
       </c>
       <c r="K84" s="14" t="n">
         <v>0</v>
@@ -4161,10 +4159,10 @@
       </c>
       <c r="E85" s="5" t="n">
         <f aca="false">SUM(F85:H85)</f>
-        <v>0.01</v>
+        <v>0.00544800000000123</v>
       </c>
       <c r="F85" s="6" t="n">
-        <v>0.01</v>
+        <v>0.00544800000000123</v>
       </c>
       <c r="G85" s="6" t="n">
         <v>0</v>
@@ -4176,7 +4174,7 @@
         <v>35</v>
       </c>
       <c r="J85" s="6" t="n">
-        <v>0.01</v>
+        <v>0.00544800000000123</v>
       </c>
       <c r="K85" s="18" t="s">
         <v>76</v>
@@ -4197,10 +4195,10 @@
       </c>
       <c r="E86" s="5" t="n">
         <f aca="false">SUM(F86:H86)</f>
-        <v>51.75</v>
+        <v>51.75348</v>
       </c>
       <c r="F86" s="6" t="n">
-        <v>51.75</v>
+        <v>51.75348</v>
       </c>
       <c r="G86" s="6" t="n">
         <v>0</v>
@@ -4212,7 +4210,7 @@
         <v>34</v>
       </c>
       <c r="J86" s="6" t="n">
-        <v>51.75</v>
+        <v>51.75348</v>
       </c>
       <c r="K86" s="18" t="s">
         <v>76</v>
@@ -4233,10 +4231,10 @@
       </c>
       <c r="E87" s="5" t="n">
         <f aca="false">SUM(F87:H87)</f>
-        <v>15.32</v>
+        <v>15.31896</v>
       </c>
       <c r="F87" s="6" t="n">
-        <v>15.32</v>
+        <v>15.31896</v>
       </c>
       <c r="G87" s="6" t="n">
         <v>0</v>
@@ -4248,7 +4246,7 @@
         <v>34</v>
       </c>
       <c r="J87" s="6" t="n">
-        <v>15.32</v>
+        <v>15.31896</v>
       </c>
       <c r="K87" s="18" t="s">
         <v>76</v>
@@ -4269,10 +4267,10 @@
       </c>
       <c r="E88" s="5" t="n">
         <f aca="false">SUM(F88:H88)</f>
-        <v>5.39</v>
+        <v>5.3884585</v>
       </c>
       <c r="F88" s="6" t="n">
-        <v>5.39</v>
+        <v>5.3884585</v>
       </c>
       <c r="G88" s="6" t="n">
         <v>0</v>
@@ -4284,7 +4282,7 @@
         <v>32</v>
       </c>
       <c r="J88" s="6" t="n">
-        <v>5.39</v>
+        <v>5.3884585</v>
       </c>
       <c r="K88" s="18" t="s">
         <v>76</v>
@@ -4305,10 +4303,10 @@
       </c>
       <c r="E89" s="5" t="n">
         <f aca="false">SUM(F89:H89)</f>
-        <v>2.01</v>
+        <v>2.00522</v>
       </c>
       <c r="F89" s="6" t="n">
-        <v>2.01</v>
+        <v>2.00522</v>
       </c>
       <c r="G89" s="6" t="n">
         <v>0</v>
@@ -4320,7 +4318,7 @@
         <v>37</v>
       </c>
       <c r="J89" s="6" t="n">
-        <v>2.01</v>
+        <v>2.00522</v>
       </c>
       <c r="K89" s="18" t="s">
         <v>76</v>
@@ -4341,10 +4339,10 @@
       </c>
       <c r="E90" s="5" t="n">
         <f aca="false">SUM(F90:H90)</f>
-        <v>0.54</v>
+        <v>0.535804799999998</v>
       </c>
       <c r="F90" s="6" t="n">
-        <v>0.54</v>
+        <v>0.535804799999998</v>
       </c>
       <c r="G90" s="6" t="n">
         <v>0</v>
@@ -4356,7 +4354,7 @@
         <v>37</v>
       </c>
       <c r="J90" s="6" t="n">
-        <v>0.54</v>
+        <v>0.535804799999998</v>
       </c>
       <c r="K90" s="18" t="s">
         <v>76</v>
@@ -4377,10 +4375,10 @@
       </c>
       <c r="E91" s="5" t="n">
         <f aca="false">SUM(F91:H91)</f>
-        <v>0.33</v>
+        <v>0.333020799999996</v>
       </c>
       <c r="F91" s="6" t="n">
-        <v>0.33</v>
+        <v>0.333020799999996</v>
       </c>
       <c r="G91" s="6" t="n">
         <v>0</v>
@@ -4392,7 +4390,7 @@
         <v>54</v>
       </c>
       <c r="J91" s="6" t="n">
-        <v>0.33</v>
+        <v>0.333020799999996</v>
       </c>
       <c r="K91" s="14" t="n">
         <v>0</v>
@@ -4413,10 +4411,10 @@
       </c>
       <c r="E92" s="5" t="n">
         <f aca="false">SUM(F92:H92)</f>
-        <v>0.27</v>
+        <v>0.267739999999995</v>
       </c>
       <c r="F92" s="6" t="n">
-        <v>0.27</v>
+        <v>0.267739999999995</v>
       </c>
       <c r="G92" s="6" t="n">
         <v>0</v>
@@ -4428,7 +4426,7 @@
         <v>37</v>
       </c>
       <c r="J92" s="6" t="n">
-        <v>0.27</v>
+        <v>0.267739999999995</v>
       </c>
       <c r="K92" s="18" t="s">
         <v>76</v>
@@ -4443,24 +4441,24 @@
       </c>
       <c r="E93" s="8" t="n">
         <f aca="false">SUBTOTAL(9,E5:E92)</f>
-        <v>757.34</v>
+        <v>757.350399642613</v>
       </c>
       <c r="F93" s="8" t="n">
         <f aca="false">SUBTOTAL(9,F5:F92)</f>
-        <v>457.05</v>
+        <v>457.034572318575</v>
       </c>
       <c r="G93" s="8" t="n">
         <f aca="false">SUBTOTAL(9,G5:G92)</f>
-        <v>50.49</v>
+        <v>50.4890326755662</v>
       </c>
       <c r="H93" s="8" t="n">
         <f aca="false">SUBTOTAL(9,H5:H92)</f>
-        <v>249.8</v>
+        <v>249.826794648472</v>
       </c>
       <c r="I93" s="19"/>
       <c r="J93" s="8" t="n">
         <f aca="false">SUBTOTAL(9,J5:J92)</f>
-        <v>1104.59</v>
+        <v>1104.59369281114</v>
       </c>
       <c r="K93" s="19"/>
     </row>
@@ -4502,11 +4500,6 @@
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="9" t="s">
         <v>123</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="9" t="s">
-        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>